<commit_message>
Add constraint of minimum allowed renewables in 2035
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52485F27-B929-4917-B544-8B3D23B3A785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6F2EE2-3939-45DF-A41A-9595D14FDBC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="100">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -331,6 +331,12 @@
   </si>
   <si>
     <t>distr*</t>
+  </si>
+  <si>
+    <t>solar,windon,windoff,geothermal,bioenergy</t>
+  </si>
+  <si>
+    <t>PP_RENEW</t>
   </si>
 </sst>
 </file>
@@ -724,25 +730,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB068F12-506D-4B74-BF24-03EBDA23C84D}">
   <dimension ref="A1:K37"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.53125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.86328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.19921875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.59765625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.3984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -768,7 +774,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B3" t="str">
         <f>"e_*"&amp;K3</f>
         <v>e_*220</v>
@@ -781,7 +787,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B4" t="str">
         <f t="shared" ref="B4:B23" si="1">"e_*"&amp;K4</f>
         <v>e_*400</v>
@@ -794,7 +800,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B5" t="str">
         <f t="shared" si="1"/>
         <v>e_*380</v>
@@ -807,7 +813,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B6" t="str">
         <f t="shared" si="1"/>
         <v>e_*225</v>
@@ -820,7 +826,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B7" t="str">
         <f t="shared" si="1"/>
         <v>e_*330</v>
@@ -833,7 +839,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B8" t="str">
         <f t="shared" si="1"/>
         <v>e_*275</v>
@@ -846,7 +852,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B9" t="str">
         <f t="shared" si="1"/>
         <v>e_*420</v>
@@ -859,7 +865,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B10" t="str">
         <f t="shared" si="1"/>
         <v>e_*300</v>
@@ -872,7 +878,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B11" t="str">
         <f t="shared" si="1"/>
         <v>e_*500</v>
@@ -885,7 +891,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B12" t="str">
         <f t="shared" si="1"/>
         <v>e_*750</v>
@@ -898,7 +904,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B13" t="str">
         <f t="shared" si="1"/>
         <v>e_*450</v>
@@ -911,7 +917,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B14" t="str">
         <f t="shared" si="1"/>
         <v>e_*515</v>
@@ -924,7 +930,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
         <f t="shared" si="1"/>
         <v>e_*525</v>
@@ -937,7 +943,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B16" t="str">
         <f t="shared" si="1"/>
         <v>e_*320</v>
@@ -950,7 +956,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
         <f t="shared" si="1"/>
         <v>e_*150</v>
@@ -963,7 +969,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B18" t="str">
         <f t="shared" si="1"/>
         <v>e_*270</v>
@@ -976,7 +982,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B19" t="str">
         <f t="shared" si="1"/>
         <v>e_*350</v>
@@ -989,7 +995,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B20" t="str">
         <f t="shared" si="1"/>
         <v>e_*250</v>
@@ -1002,7 +1008,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B21" t="str">
         <f t="shared" si="1"/>
         <v>e_*200</v>
@@ -1015,7 +1021,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B22" t="str">
         <f t="shared" si="1"/>
         <v>e_*236</v>
@@ -1028,7 +1034,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" t="str">
         <f t="shared" si="1"/>
         <v>e_*600</v>
@@ -1041,7 +1047,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>51</v>
       </c>
@@ -1049,7 +1055,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>52</v>
       </c>
@@ -1057,7 +1063,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>67</v>
       </c>
@@ -1065,7 +1071,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>68</v>
       </c>
@@ -1073,7 +1079,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>53</v>
       </c>
@@ -1082,7 +1088,7 @@
         <v>bioenergy</v>
       </c>
     </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>54</v>
       </c>
@@ -1091,7 +1097,7 @@
         <v>hydrogen</v>
       </c>
     </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>43</v>
       </c>
@@ -1100,7 +1106,7 @@
         <v>nuclear</v>
       </c>
     </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>55</v>
       </c>
@@ -1109,7 +1115,7 @@
         <v>ELC</v>
       </c>
     </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>56</v>
       </c>
@@ -1117,7 +1123,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>57</v>
       </c>
@@ -1125,7 +1131,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>58</v>
       </c>
@@ -1133,7 +1139,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>59</v>
       </c>
@@ -1141,7 +1147,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>60</v>
       </c>
@@ -1150,7 +1156,7 @@
         <v>co2</v>
       </c>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>61</v>
       </c>
@@ -1169,22 +1175,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71754C8A-E599-4286-919F-11B5789CC171}">
-  <dimension ref="A1:K48"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:K49"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="86" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.3984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.59765625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.86328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1216,7 +1223,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>29</v>
       </c>
@@ -1233,7 +1240,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>22</v>
       </c>
@@ -1241,7 +1248,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>23</v>
       </c>
@@ -1249,7 +1256,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>30</v>
       </c>
@@ -1263,7 +1270,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>31</v>
       </c>
@@ -1271,7 +1278,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>33</v>
       </c>
@@ -1279,7 +1286,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>32</v>
       </c>
@@ -1287,7 +1294,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>28</v>
       </c>
@@ -1295,7 +1302,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
         <v>40</v>
       </c>
@@ -1303,7 +1310,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3"/>
       <c r="D12" t="s">
         <v>91</v>
@@ -1315,7 +1322,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
         <v>92</v>
       </c>
@@ -1326,7 +1333,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
         <v>41</v>
       </c>
@@ -1334,7 +1341,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -1348,7 +1355,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -1362,7 +1369,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>79</v>
       </c>
@@ -1379,7 +1386,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>77</v>
       </c>
@@ -1390,7 +1397,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -1401,7 +1408,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1418,7 +1425,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -1429,7 +1436,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>47</v>
       </c>
@@ -1440,7 +1447,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -1448,7 +1455,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -1459,7 +1466,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>69</v>
       </c>
@@ -1470,7 +1477,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B26" t="str">
         <f>"g[_]*"&amp;K26</f>
         <v>g[_]*220</v>
@@ -1483,7 +1490,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B27" t="str">
         <f t="shared" ref="B27:B46" si="0">"g[_]*"&amp;K27</f>
         <v>g[_]*400</v>
@@ -1496,7 +1503,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*380</v>
@@ -1509,7 +1516,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*225</v>
@@ -1522,7 +1529,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B30" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*330</v>
@@ -1535,7 +1542,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*275</v>
@@ -1548,7 +1555,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B32" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*420</v>
@@ -1561,7 +1568,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B33" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*300</v>
@@ -1574,7 +1581,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B34" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*500</v>
@@ -1587,7 +1594,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B35" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*750</v>
@@ -1600,7 +1607,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B36" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*450</v>
@@ -1613,7 +1620,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B37" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*515</v>
@@ -1626,7 +1633,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B38" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*525</v>
@@ -1639,7 +1646,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B39" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*320</v>
@@ -1652,7 +1659,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*150</v>
@@ -1665,7 +1672,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B41" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*270</v>
@@ -1678,7 +1685,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*350</v>
@@ -1691,7 +1698,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*250</v>
@@ -1704,7 +1711,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B44" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*200</v>
@@ -1717,7 +1724,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B45" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*236</v>
@@ -1730,7 +1737,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B46" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*600</v>
@@ -1743,7 +1750,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
         <v>97</v>
       </c>
@@ -1751,12 +1758,23 @@
         <v>85</v>
       </c>
     </row>
-    <row r="48" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>86</v>
       </c>
       <c r="F48" t="s">
         <v>87</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>11</v>
+      </c>
+      <c r="D49" t="s">
+        <v>98</v>
+      </c>
+      <c r="F49" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix constraint of renewable production
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6F2EE2-3939-45DF-A41A-9595D14FDBC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93841E10-EC32-485F-9513-A95D09B9EFD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -333,10 +333,10 @@
     <t>distr*</t>
   </si>
   <si>
-    <t>solar,windon,windoff,geothermal,bioenergy</t>
-  </si>
-  <si>
     <t>PP_RENEW</t>
+  </si>
+  <si>
+    <t>Solar elec,Wind elec,geothermal,bioenergy</t>
   </si>
 </sst>
 </file>
@@ -730,25 +730,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB068F12-506D-4B74-BF24-03EBDA23C84D}">
   <dimension ref="A1:K37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -774,7 +774,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B3" t="str">
         <f>"e_*"&amp;K3</f>
         <v>e_*220</v>
@@ -787,7 +787,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B4" t="str">
         <f t="shared" ref="B4:B23" si="1">"e_*"&amp;K4</f>
         <v>e_*400</v>
@@ -800,7 +800,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B5" t="str">
         <f t="shared" si="1"/>
         <v>e_*380</v>
@@ -813,7 +813,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B6" t="str">
         <f t="shared" si="1"/>
         <v>e_*225</v>
@@ -826,7 +826,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B7" t="str">
         <f t="shared" si="1"/>
         <v>e_*330</v>
@@ -839,7 +839,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B8" t="str">
         <f t="shared" si="1"/>
         <v>e_*275</v>
@@ -852,7 +852,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B9" t="str">
         <f t="shared" si="1"/>
         <v>e_*420</v>
@@ -865,7 +865,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B10" t="str">
         <f t="shared" si="1"/>
         <v>e_*300</v>
@@ -878,7 +878,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B11" t="str">
         <f t="shared" si="1"/>
         <v>e_*500</v>
@@ -891,7 +891,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B12" t="str">
         <f t="shared" si="1"/>
         <v>e_*750</v>
@@ -904,7 +904,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B13" t="str">
         <f t="shared" si="1"/>
         <v>e_*450</v>
@@ -917,7 +917,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B14" t="str">
         <f t="shared" si="1"/>
         <v>e_*515</v>
@@ -930,7 +930,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B15" t="str">
         <f t="shared" si="1"/>
         <v>e_*525</v>
@@ -943,7 +943,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B16" t="str">
         <f t="shared" si="1"/>
         <v>e_*320</v>
@@ -956,7 +956,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B17" t="str">
         <f t="shared" si="1"/>
         <v>e_*150</v>
@@ -969,7 +969,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B18" t="str">
         <f t="shared" si="1"/>
         <v>e_*270</v>
@@ -982,7 +982,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B19" t="str">
         <f t="shared" si="1"/>
         <v>e_*350</v>
@@ -995,7 +995,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B20" t="str">
         <f t="shared" si="1"/>
         <v>e_*250</v>
@@ -1008,7 +1008,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B21" t="str">
         <f t="shared" si="1"/>
         <v>e_*200</v>
@@ -1021,7 +1021,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B22" t="str">
         <f t="shared" si="1"/>
         <v>e_*236</v>
@@ -1034,7 +1034,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B23" t="str">
         <f t="shared" si="1"/>
         <v>e_*600</v>
@@ -1047,7 +1047,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>51</v>
       </c>
@@ -1055,7 +1055,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>52</v>
       </c>
@@ -1063,7 +1063,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>67</v>
       </c>
@@ -1071,7 +1071,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>68</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>53</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>bioenergy</v>
       </c>
     </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
         <v>54</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>hydrogen</v>
       </c>
     </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>43</v>
       </c>
@@ -1106,7 +1106,7 @@
         <v>nuclear</v>
       </c>
     </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
         <v>55</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>ELC</v>
       </c>
     </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
         <v>56</v>
       </c>
@@ -1123,7 +1123,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
         <v>57</v>
       </c>
@@ -1131,7 +1131,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B34" t="s">
         <v>58</v>
       </c>
@@ -1139,7 +1139,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B35" t="s">
         <v>59</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B36" t="s">
         <v>60</v>
       </c>
@@ -1156,7 +1156,7 @@
         <v>co2</v>
       </c>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B37" t="s">
         <v>61</v>
       </c>
@@ -1176,22 +1176,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71754C8A-E599-4286-919F-11B5789CC171}">
   <dimension ref="A1:K49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="86" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="17.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1223,7 +1223,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>29</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>22</v>
       </c>
@@ -1248,7 +1248,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>23</v>
       </c>
@@ -1256,7 +1256,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>30</v>
       </c>
@@ -1270,7 +1270,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>31</v>
       </c>
@@ -1278,7 +1278,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>33</v>
       </c>
@@ -1286,7 +1286,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>32</v>
       </c>
@@ -1294,7 +1294,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>28</v>
       </c>
@@ -1302,7 +1302,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D11" t="s">
         <v>40</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B12" s="3"/>
       <c r="D12" t="s">
         <v>91</v>
@@ -1322,7 +1322,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D13" t="s">
         <v>92</v>
       </c>
@@ -1333,7 +1333,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D14" t="s">
         <v>41</v>
       </c>
@@ -1341,7 +1341,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -1355,7 +1355,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -1369,7 +1369,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
         <v>79</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>77</v>
       </c>
@@ -1397,7 +1397,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1425,7 +1425,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>47</v>
       </c>
@@ -1447,7 +1447,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -1455,7 +1455,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -1466,7 +1466,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>69</v>
       </c>
@@ -1477,7 +1477,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B26" t="str">
         <f>"g[_]*"&amp;K26</f>
         <v>g[_]*220</v>
@@ -1490,7 +1490,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B27" t="str">
         <f t="shared" ref="B27:B46" si="0">"g[_]*"&amp;K27</f>
         <v>g[_]*400</v>
@@ -1503,7 +1503,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*380</v>
@@ -1516,7 +1516,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*225</v>
@@ -1529,7 +1529,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B30" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*330</v>
@@ -1542,7 +1542,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*275</v>
@@ -1555,7 +1555,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B32" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*420</v>
@@ -1568,7 +1568,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B33" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*300</v>
@@ -1581,7 +1581,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B34" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*500</v>
@@ -1594,7 +1594,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B35" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*750</v>
@@ -1607,7 +1607,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B36" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*450</v>
@@ -1620,7 +1620,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B37" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*515</v>
@@ -1633,7 +1633,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B38" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*525</v>
@@ -1646,7 +1646,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B39" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*320</v>
@@ -1659,7 +1659,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B40" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*150</v>
@@ -1672,7 +1672,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B41" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*270</v>
@@ -1685,7 +1685,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B42" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*350</v>
@@ -1698,7 +1698,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B43" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*250</v>
@@ -1711,7 +1711,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B44" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*200</v>
@@ -1724,7 +1724,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B45" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*236</v>
@@ -1737,7 +1737,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B46" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*600</v>
@@ -1750,7 +1750,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B47" t="s">
         <v>97</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="48" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B48" t="s">
         <v>86</v>
       </c>
@@ -1766,15 +1766,15 @@
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>11</v>
       </c>
       <c r="D49" t="s">
+        <v>99</v>
+      </c>
+      <c r="F49" t="s">
         <v>98</v>
-      </c>
-      <c r="F49" t="s">
-        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Attempt 2: Fix constraint of renewable production
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93841E10-EC32-485F-9513-A95D09B9EFD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3182BF65-8F72-49C8-9499-D8546BD20251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -336,7 +336,7 @@
     <t>PP_RENEW</t>
   </si>
   <si>
-    <t>Solar elec,Wind elec,geothermal,bioenergy</t>
+    <t>renewable, bioenergy</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Attempt 2.1: Fix constraint of renewable production
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3182BF65-8F72-49C8-9499-D8546BD20251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74870EF3-B698-4D2F-B557-AE39410E1825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="99">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -334,9 +334,6 @@
   </si>
   <si>
     <t>PP_RENEW</t>
-  </si>
-  <si>
-    <t>renewable, bioenergy</t>
   </si>
 </sst>
 </file>
@@ -1771,7 +1768,7 @@
         <v>11</v>
       </c>
       <c r="D49" t="s">
-        <v>99</v>
+        <v>43</v>
       </c>
       <c r="F49" t="s">
         <v>98</v>

</xml_diff>

<commit_message>
Attempt 3: Fix constraint of renewable production
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74870EF3-B698-4D2F-B557-AE39410E1825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E1D6BB-8FF5-4AC0-B603-F17CF3FE60DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="100">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -334,6 +334,9 @@
   </si>
   <si>
     <t>PP_RENEW</t>
+  </si>
+  <si>
+    <t>renewable,bioenergy</t>
   </si>
 </sst>
 </file>
@@ -1768,7 +1771,7 @@
         <v>11</v>
       </c>
       <c r="D49" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="F49" t="s">
         <v>98</v>

</xml_diff>

<commit_message>
Attempt 5: Fix constraint of renewable production
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF16F568-7F4A-44C5-9E13-F86C0A7C2D25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1441EDD-8D2D-4E3B-BAA4-5C4AB5190B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -336,7 +336,7 @@
     <t>PP_RENEW</t>
   </si>
   <si>
-    <t>renewable,bioenergy</t>
+    <t>geothermal,hydro,solar,wind,bioenergy</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Attempt 6: Fix constraint of renewable production
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1441EDD-8D2D-4E3B-BAA4-5C4AB5190B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57B80DD2-3B90-47A4-A1DF-DB3C8016F842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -336,7 +336,7 @@
     <t>PP_RENEW</t>
   </si>
   <si>
-    <t>geothermal,hydro,solar,wind,bioenergy</t>
+    <t>geothermal,hydro,solar,windon,windoff,bioenergy</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Attempt 7: Fix constraint of renewable production
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57B80DD2-3B90-47A4-A1DF-DB3C8016F842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68B5E479-DE6C-490F-8BA9-757ED633082E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -336,7 +336,7 @@
     <t>PP_RENEW</t>
   </si>
   <si>
-    <t>geothermal,hydro,solar,windon,windoff,bioenergy</t>
+    <t>geothermal,hydro,e*spv*,e*won*,e*wof*,bioenergy</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Testing solid power plants constraint
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68B5E479-DE6C-490F-8BA9-757ED633082E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FABAAD33-7564-410B-8F55-7E1328167797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="102">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -337,6 +337,12 @@
   </si>
   <si>
     <t>geothermal,hydro,e*spv*,e*won*,e*wof*,bioenergy</t>
+  </si>
+  <si>
+    <t>solid</t>
+  </si>
+  <si>
+    <t>coal,gas,oil,bioenery,hydrogen,nuclear</t>
   </si>
 </sst>
 </file>
@@ -729,11 +735,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB068F12-506D-4B74-BF24-03EBDA23C84D}">
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.81640625" bestFit="1" customWidth="1"/>
@@ -1163,6 +1169,14 @@
       <c r="D37" t="str">
         <f>B37</f>
         <v>co2captured</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B38" t="s">
+        <v>101</v>
+      </c>
+      <c r="D38" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Attemps 3: Testing solid power plants constraint
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FABAAD33-7564-410B-8F55-7E1328167797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{372C8863-25E4-4E5E-9662-D7E605C1043C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="104">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -343,6 +343,12 @@
   </si>
   <si>
     <t>coal,gas,oil,bioenery,hydrogen,nuclear</t>
+  </si>
+  <si>
+    <t>pp_controllable</t>
+  </si>
+  <si>
+    <t>geothermal,hydro,bioenergy,nuclear,fossil,</t>
   </si>
 </sst>
 </file>
@@ -1189,12 +1195,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71754C8A-E599-4286-919F-11B5789CC171}">
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="86" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="41.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.81640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.453125" bestFit="1" customWidth="1"/>
@@ -1791,6 +1797,14 @@
         <v>98</v>
       </c>
     </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D50" t="s">
+        <v>103</v>
+      </c>
+      <c r="F50" t="s">
+        <v>102</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Attemps 5: Testing solid power plants constraint
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{372C8863-25E4-4E5E-9662-D7E605C1043C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FC49EF-1F11-461F-98DC-9F8E02A5B60A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -348,7 +348,7 @@
     <t>pp_controllable</t>
   </si>
   <si>
-    <t>geothermal,hydro,bioenergy,nuclear,fossil,</t>
+    <t>geothermal,hydro,bioenergy,GAS,OIL,nuclear</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Changing renewable penetration constraint logic part 6
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/Sets-vervestacks.xlsx
+++ b/VerveStacks_EST/Sets-vervestacks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FC49EF-1F11-461F-98DC-9F8E02A5B60A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB98498B-D954-46FC-94A2-48ED9BDAEFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -348,7 +348,7 @@
     <t>pp_controllable</t>
   </si>
   <si>
-    <t>geothermal,hydro,bioenergy,GAS,OIL,nuclear</t>
+    <t>geothermal,hydro,bioenergy,GAS,OIL,nuclear, COAL</t>
   </si>
 </sst>
 </file>
@@ -742,25 +742,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB068F12-506D-4B74-BF24-03EBDA23C84D}">
   <dimension ref="A1:K38"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -786,7 +786,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B3" t="str">
         <f>"e_*"&amp;K3</f>
         <v>e_*220</v>
@@ -799,7 +799,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B4" t="str">
         <f t="shared" ref="B4:B23" si="1">"e_*"&amp;K4</f>
         <v>e_*400</v>
@@ -812,7 +812,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B5" t="str">
         <f t="shared" si="1"/>
         <v>e_*380</v>
@@ -825,7 +825,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B6" t="str">
         <f t="shared" si="1"/>
         <v>e_*225</v>
@@ -838,7 +838,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B7" t="str">
         <f t="shared" si="1"/>
         <v>e_*330</v>
@@ -851,7 +851,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B8" t="str">
         <f t="shared" si="1"/>
         <v>e_*275</v>
@@ -864,7 +864,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B9" t="str">
         <f t="shared" si="1"/>
         <v>e_*420</v>
@@ -877,7 +877,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B10" t="str">
         <f t="shared" si="1"/>
         <v>e_*300</v>
@@ -890,7 +890,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B11" t="str">
         <f t="shared" si="1"/>
         <v>e_*500</v>
@@ -903,7 +903,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B12" t="str">
         <f t="shared" si="1"/>
         <v>e_*750</v>
@@ -916,7 +916,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B13" t="str">
         <f t="shared" si="1"/>
         <v>e_*450</v>
@@ -929,7 +929,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B14" t="str">
         <f t="shared" si="1"/>
         <v>e_*515</v>
@@ -942,7 +942,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
         <f t="shared" si="1"/>
         <v>e_*525</v>
@@ -955,7 +955,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B16" t="str">
         <f t="shared" si="1"/>
         <v>e_*320</v>
@@ -968,7 +968,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
         <f t="shared" si="1"/>
         <v>e_*150</v>
@@ -981,7 +981,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B18" t="str">
         <f t="shared" si="1"/>
         <v>e_*270</v>
@@ -994,7 +994,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B19" t="str">
         <f t="shared" si="1"/>
         <v>e_*350</v>
@@ -1007,7 +1007,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B20" t="str">
         <f t="shared" si="1"/>
         <v>e_*250</v>
@@ -1020,7 +1020,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B21" t="str">
         <f t="shared" si="1"/>
         <v>e_*200</v>
@@ -1033,7 +1033,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B22" t="str">
         <f t="shared" si="1"/>
         <v>e_*236</v>
@@ -1046,7 +1046,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" t="str">
         <f t="shared" si="1"/>
         <v>e_*600</v>
@@ -1059,7 +1059,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>51</v>
       </c>
@@ -1067,7 +1067,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>52</v>
       </c>
@@ -1075,7 +1075,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>67</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>68</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>53</v>
       </c>
@@ -1100,7 +1100,7 @@
         <v>bioenergy</v>
       </c>
     </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>54</v>
       </c>
@@ -1109,7 +1109,7 @@
         <v>hydrogen</v>
       </c>
     </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>43</v>
       </c>
@@ -1118,7 +1118,7 @@
         <v>nuclear</v>
       </c>
     </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>55</v>
       </c>
@@ -1127,7 +1127,7 @@
         <v>ELC</v>
       </c>
     </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>56</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>57</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>58</v>
       </c>
@@ -1151,7 +1151,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>59</v>
       </c>
@@ -1159,7 +1159,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>60</v>
       </c>
@@ -1168,7 +1168,7 @@
         <v>co2</v>
       </c>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>61</v>
       </c>
@@ -1177,7 +1177,7 @@
         <v>co2captured</v>
       </c>
     </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>101</v>
       </c>
@@ -1196,22 +1196,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71754C8A-E599-4286-919F-11B5789CC171}">
   <dimension ref="A1:K50"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="86" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1243,7 +1243,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>29</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>22</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>23</v>
       </c>
@@ -1276,7 +1276,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>30</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>31</v>
       </c>
@@ -1298,7 +1298,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>33</v>
       </c>
@@ -1306,7 +1306,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>32</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>28</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
         <v>40</v>
       </c>
@@ -1330,7 +1330,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B12" s="3"/>
       <c r="D12" t="s">
         <v>91</v>
@@ -1342,7 +1342,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
         <v>92</v>
       </c>
@@ -1353,7 +1353,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
         <v>41</v>
       </c>
@@ -1361,7 +1361,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -1375,7 +1375,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -1389,7 +1389,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>79</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>77</v>
       </c>
@@ -1417,7 +1417,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -1428,7 +1428,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1445,7 +1445,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -1456,7 +1456,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>47</v>
       </c>
@@ -1467,7 +1467,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -1475,7 +1475,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -1486,7 +1486,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>69</v>
       </c>
@@ -1497,7 +1497,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B26" t="str">
         <f>"g[_]*"&amp;K26</f>
         <v>g[_]*220</v>
@@ -1510,7 +1510,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B27" t="str">
         <f t="shared" ref="B27:B46" si="0">"g[_]*"&amp;K27</f>
         <v>g[_]*400</v>
@@ -1523,7 +1523,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*380</v>
@@ -1536,7 +1536,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*225</v>
@@ -1549,7 +1549,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B30" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*330</v>
@@ -1562,7 +1562,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*275</v>
@@ -1575,7 +1575,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B32" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*420</v>
@@ -1588,7 +1588,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B33" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*300</v>
@@ -1601,7 +1601,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B34" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*500</v>
@@ -1614,7 +1614,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B35" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*750</v>
@@ -1627,7 +1627,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B36" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*450</v>
@@ -1640,7 +1640,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B37" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*515</v>
@@ -1653,7 +1653,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B38" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*525</v>
@@ -1666,7 +1666,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B39" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*320</v>
@@ -1679,7 +1679,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*150</v>
@@ -1692,7 +1692,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B41" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*270</v>
@@ -1705,7 +1705,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*350</v>
@@ -1718,7 +1718,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*250</v>
@@ -1731,7 +1731,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B44" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*200</v>
@@ -1744,7 +1744,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B45" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*236</v>
@@ -1757,7 +1757,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B46" t="str">
         <f t="shared" si="0"/>
         <v>g[_]*600</v>
@@ -1770,7 +1770,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
         <v>97</v>
       </c>
@@ -1778,7 +1778,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="48" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>86</v>
       </c>
@@ -1786,7 +1786,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>11</v>
       </c>
@@ -1797,7 +1797,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D50" t="s">
         <v>103</v>
       </c>

</xml_diff>